<commit_message>
feat(extractores): elimina el extractor HTML, formato ausente del corpus real
El corpus real de ADL no trae archivos .html/.htm, así que mantener el
extractor y su registro en EXTRACTORES/FORMATOS era complejidad muerta que
arrastraba dependencias (beautifulsoup4, lxml) y fixtures sin ningún archivo
real que las ejercitara.

- Borra extractores/html.py y tests/test_html.py.
- Quita .html/.htm de EXTRACTORES (orquestador.py) y "html" de FORMATOS
  (contrato.py).
- Las fixtures y pruebas de orquestador/índice que usaban .html solo como
  formato genérico de prueba pasan a .txt, que sí existe en el corpus real.
- Actualiza README y docstrings que documentaban a html.py como
  implementación de referencia.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRTzuXe39V3sxrLLaWmYaU
</commit_message>
<xml_diff>
--- a/fixtures/indice_minimo.xlsx
+++ b/fixtures/indice_minimo.xlsx
@@ -476,13 +476,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>bien_formado.html</t>
+          <t>bien_formado.txt</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>TXT</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>informe.html</t>
+          <t>informe.txt</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>TXT</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>informe.html</t>
+          <t>informe.txt</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>TXT</t>
         </is>
       </c>
     </row>
@@ -583,13 +583,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>anidado.html</t>
+          <t>anidado.txt</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>TXT</t>
         </is>
       </c>
     </row>

</xml_diff>